<commit_message>
Added evacuation dates, start/end times to inventory creation code
Also fixed pooled sample inventory - samples pooled over multiple days.
</commit_message>
<xml_diff>
--- a/processing_scripts/Inventory_Processing/TEMPEST_Porewater_pH_updated.xlsx
+++ b/processing_scripts/Inventory_Processing/TEMPEST_Porewater_pH_updated.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="225">
   <si>
     <t>Site</t>
   </si>
@@ -683,6 +683,9 @@
     <t xml:space="preserve">no cond value entered on data sheet</t>
   </si>
   <si>
+    <t xml:space="preserve">Oakton</t>
+  </si>
+  <si>
     <t xml:space="preserve">cloudy; colloids??</t>
   </si>
   <si>
@@ -39597,35 +39600,39 @@
         <v>136</v>
       </c>
       <c r="C919" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="D919" t="n">
         <v>50</v>
       </c>
-      <c r="E919"/>
+      <c r="E919" t="n">
+        <v>20260810</v>
+      </c>
       <c r="F919" t="n">
-        <v>835</v>
+        <v>1420</v>
       </c>
       <c r="G919" t="s">
         <v>138</v>
       </c>
       <c r="H919" t="n">
-        <v>6.93</v>
+        <v>6.26</v>
       </c>
       <c r="I919" t="n">
-        <v>124.9</v>
-      </c>
-      <c r="J919"/>
+        <v>17</v>
+      </c>
+      <c r="J919" t="s">
+        <v>176</v>
+      </c>
       <c r="K919" t="n">
-        <v>24.9</v>
+        <v>29.9</v>
       </c>
       <c r="L919" t="s">
         <v>140</v>
       </c>
-      <c r="M919"/>
-      <c r="N919" t="s">
+      <c r="M919" t="s">
         <v>222</v>
       </c>
+      <c r="N919"/>
       <c r="O919"/>
     </row>
     <row r="920">
@@ -39636,32 +39643,38 @@
         <v>136</v>
       </c>
       <c r="C920" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D920" t="n">
+        <v>15</v>
+      </c>
+      <c r="E920" t="n">
+        <v>20260810</v>
+      </c>
+      <c r="F920" t="n">
+        <v>1425</v>
+      </c>
+      <c r="G920" t="s">
+        <v>138</v>
+      </c>
+      <c r="H920" t="n">
+        <v>6.34</v>
+      </c>
+      <c r="I920" t="n">
+        <v>5.59</v>
+      </c>
+      <c r="J920" t="s">
+        <v>176</v>
+      </c>
+      <c r="K920" t="n">
         <v>30</v>
       </c>
-      <c r="E920"/>
-      <c r="F920" t="n">
-        <v>820</v>
-      </c>
-      <c r="G920" t="s">
-        <v>138</v>
-      </c>
-      <c r="H920" t="n">
-        <v>7.08</v>
-      </c>
-      <c r="I920" t="n">
-        <v>100.1</v>
-      </c>
-      <c r="J920"/>
-      <c r="K920" t="n">
-        <v>24.9</v>
-      </c>
       <c r="L920" t="s">
         <v>140</v>
       </c>
-      <c r="M920"/>
+      <c r="M920" t="s">
+        <v>222</v>
+      </c>
       <c r="N920"/>
       <c r="O920"/>
     </row>
@@ -39670,35 +39683,41 @@
         <v>135</v>
       </c>
       <c r="B921" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C921" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D921" t="n">
-        <v>50</v>
-      </c>
-      <c r="E921"/>
+        <v>30</v>
+      </c>
+      <c r="E921" t="n">
+        <v>20260810</v>
+      </c>
       <c r="F921" t="n">
-        <v>1420</v>
+        <v>1310</v>
       </c>
       <c r="G921" t="s">
         <v>138</v>
       </c>
       <c r="H921" t="n">
-        <v>6.26</v>
+        <v>4.35</v>
       </c>
       <c r="I921" t="n">
-        <v>17</v>
-      </c>
-      <c r="J921"/>
+        <v>5.4</v>
+      </c>
+      <c r="J921" t="s">
+        <v>176</v>
+      </c>
       <c r="K921" t="n">
-        <v>29.9</v>
+        <v>26.7</v>
       </c>
       <c r="L921" t="s">
         <v>140</v>
       </c>
-      <c r="M921"/>
+      <c r="M921" t="s">
+        <v>222</v>
+      </c>
       <c r="N921"/>
       <c r="O921"/>
     </row>
@@ -39707,35 +39726,39 @@
         <v>135</v>
       </c>
       <c r="B922" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="C922" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="D922" t="n">
-        <v>15</v>
-      </c>
-      <c r="E922"/>
+        <v>30</v>
+      </c>
+      <c r="E922" t="n">
+        <v>20260810</v>
+      </c>
       <c r="F922" t="n">
-        <v>1425</v>
+        <v>1135</v>
       </c>
       <c r="G922" t="s">
         <v>138</v>
       </c>
       <c r="H922" t="n">
-        <v>6.34</v>
-      </c>
-      <c r="I922" t="n">
-        <v>5.59</v>
-      </c>
-      <c r="J922"/>
+        <v>5.48</v>
+      </c>
+      <c r="I922"/>
+      <c r="J922" t="s">
+        <v>176</v>
+      </c>
       <c r="K922" t="n">
-        <v>30</v>
+        <v>26.6</v>
       </c>
       <c r="L922" t="s">
-        <v>140</v>
-      </c>
-      <c r="M922"/>
+        <v>162</v>
+      </c>
+      <c r="M922" t="s">
+        <v>222</v>
+      </c>
       <c r="N922"/>
       <c r="O922"/>
     </row>
@@ -39747,35 +39770,39 @@
         <v>144</v>
       </c>
       <c r="C923" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="D923" t="n">
-        <v>15</v>
-      </c>
-      <c r="E923"/>
+        <v>30</v>
+      </c>
+      <c r="E923" t="n">
+        <v>20260810</v>
+      </c>
       <c r="F923" t="n">
-        <v>905</v>
+        <v>1248</v>
       </c>
       <c r="G923" t="s">
         <v>138</v>
       </c>
       <c r="H923" t="n">
-        <v>5.99</v>
+        <v>3.92</v>
       </c>
       <c r="I923" t="n">
-        <v>1822</v>
-      </c>
-      <c r="J923"/>
+        <v>4.4</v>
+      </c>
+      <c r="J923" t="s">
+        <v>176</v>
+      </c>
       <c r="K923" t="n">
-        <v>24.7</v>
+        <v>26.6</v>
       </c>
       <c r="L923" t="s">
-        <v>162</v>
-      </c>
-      <c r="M923"/>
-      <c r="N923" t="s">
-        <v>223</v>
-      </c>
+        <v>140</v>
+      </c>
+      <c r="M923" t="s">
+        <v>222</v>
+      </c>
+      <c r="N923"/>
       <c r="O923"/>
     </row>
     <row r="924">
@@ -39786,35 +39813,39 @@
         <v>144</v>
       </c>
       <c r="C924" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D924" t="n">
-        <v>15</v>
-      </c>
-      <c r="E924"/>
+        <v>50</v>
+      </c>
+      <c r="E924" t="n">
+        <v>20260810</v>
+      </c>
       <c r="F924" t="n">
-        <v>851</v>
+        <v>1257</v>
       </c>
       <c r="G924" t="s">
         <v>138</v>
       </c>
       <c r="H924" t="n">
-        <v>6.18</v>
+        <v>4.02</v>
       </c>
       <c r="I924" t="n">
-        <v>1752</v>
-      </c>
-      <c r="J924"/>
+        <v>4.81</v>
+      </c>
+      <c r="J924" t="s">
+        <v>176</v>
+      </c>
       <c r="K924" t="n">
-        <v>25.2</v>
+        <v>25.6</v>
       </c>
       <c r="L924" t="s">
         <v>140</v>
       </c>
-      <c r="M924"/>
-      <c r="N924" t="s">
-        <v>223</v>
-      </c>
+      <c r="M924" t="s">
+        <v>222</v>
+      </c>
+      <c r="N924"/>
       <c r="O924"/>
     </row>
     <row r="925">
@@ -39825,33 +39856,41 @@
         <v>144</v>
       </c>
       <c r="C925" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D925" t="n">
         <v>30</v>
       </c>
-      <c r="E925"/>
+      <c r="E925" t="n">
+        <v>20260810</v>
+      </c>
       <c r="F925" t="n">
-        <v>1310</v>
+        <v>1217</v>
       </c>
       <c r="G925" t="s">
         <v>138</v>
       </c>
       <c r="H925" t="n">
-        <v>4.35</v>
+        <v>4.46</v>
       </c>
       <c r="I925" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="J925"/>
+        <v>4.19</v>
+      </c>
+      <c r="J925" t="s">
+        <v>176</v>
+      </c>
       <c r="K925" t="n">
-        <v>26.7</v>
+        <v>26.2</v>
       </c>
       <c r="L925" t="s">
-        <v>140</v>
-      </c>
-      <c r="M925"/>
-      <c r="N925"/>
+        <v>162</v>
+      </c>
+      <c r="M925" t="s">
+        <v>222</v>
+      </c>
+      <c r="N925" t="s">
+        <v>223</v>
+      </c>
       <c r="O925"/>
     </row>
     <row r="926">
@@ -39862,33 +39901,41 @@
         <v>144</v>
       </c>
       <c r="C926" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D926" t="n">
         <v>50</v>
       </c>
-      <c r="E926"/>
+      <c r="E926" t="n">
+        <v>20260810</v>
+      </c>
       <c r="F926" t="n">
-        <v>854</v>
+        <v>1236</v>
       </c>
       <c r="G926" t="s">
         <v>138</v>
       </c>
       <c r="H926" t="n">
-        <v>4.28</v>
+        <v>3.75</v>
       </c>
       <c r="I926" t="n">
-        <v>6.71</v>
-      </c>
-      <c r="J926"/>
+        <v>8.54</v>
+      </c>
+      <c r="J926" t="s">
+        <v>176</v>
+      </c>
       <c r="K926" t="n">
-        <v>24.4</v>
+        <v>26.4</v>
       </c>
       <c r="L926" t="s">
-        <v>140</v>
-      </c>
-      <c r="M926"/>
-      <c r="N926"/>
+        <v>162</v>
+      </c>
+      <c r="M926" t="s">
+        <v>222</v>
+      </c>
+      <c r="N926" t="s">
+        <v>223</v>
+      </c>
       <c r="O926"/>
     </row>
     <row r="927">
@@ -39899,30 +39946,38 @@
         <v>144</v>
       </c>
       <c r="C927" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="D927" t="n">
         <v>30</v>
       </c>
-      <c r="E927"/>
+      <c r="E927" t="n">
+        <v>20260810</v>
+      </c>
       <c r="F927" t="n">
-        <v>1135</v>
+        <v>1157</v>
       </c>
       <c r="G927" t="s">
         <v>138</v>
       </c>
       <c r="H927" t="n">
-        <v>5.48</v>
-      </c>
-      <c r="I927"/>
-      <c r="J927"/>
+        <v>3.85</v>
+      </c>
+      <c r="I927" t="n">
+        <v>4.92</v>
+      </c>
+      <c r="J927" t="s">
+        <v>176</v>
+      </c>
       <c r="K927" t="n">
-        <v>26.6</v>
+        <v>26.2</v>
       </c>
       <c r="L927" t="s">
-        <v>162</v>
-      </c>
-      <c r="M927"/>
+        <v>140</v>
+      </c>
+      <c r="M927" t="s">
+        <v>222</v>
+      </c>
       <c r="N927"/>
       <c r="O927"/>
     </row>
@@ -39934,32 +39989,38 @@
         <v>144</v>
       </c>
       <c r="C928" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="D928" t="n">
         <v>50</v>
       </c>
-      <c r="E928"/>
+      <c r="E928" t="n">
+        <v>20260810</v>
+      </c>
       <c r="F928" t="n">
-        <v>915</v>
+        <v>1204</v>
       </c>
       <c r="G928" t="s">
         <v>138</v>
       </c>
       <c r="H928" t="n">
-        <v>4.6</v>
+        <v>4.03</v>
       </c>
       <c r="I928" t="n">
-        <v>3.69</v>
-      </c>
-      <c r="J928"/>
+        <v>4.35</v>
+      </c>
+      <c r="J928" t="s">
+        <v>176</v>
+      </c>
       <c r="K928" t="n">
-        <v>23.9</v>
+        <v>25.5</v>
       </c>
       <c r="L928" t="s">
         <v>140</v>
       </c>
-      <c r="M928"/>
+      <c r="M928" t="s">
+        <v>222</v>
+      </c>
       <c r="N928"/>
       <c r="O928"/>
     </row>
@@ -39968,35 +40029,41 @@
         <v>135</v>
       </c>
       <c r="B929" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C929" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="D929" t="n">
         <v>30</v>
       </c>
-      <c r="E929"/>
+      <c r="E929" t="n">
+        <v>20260810</v>
+      </c>
       <c r="F929" t="n">
-        <v>1248</v>
+        <v>1030</v>
       </c>
       <c r="G929" t="s">
         <v>138</v>
       </c>
       <c r="H929" t="n">
-        <v>3.92</v>
+        <v>5.83</v>
       </c>
       <c r="I929" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="J929"/>
+        <v>56.6</v>
+      </c>
+      <c r="J929" t="s">
+        <v>176</v>
+      </c>
       <c r="K929" t="n">
-        <v>26.6</v>
+        <v>25.3</v>
       </c>
       <c r="L929" t="s">
         <v>140</v>
       </c>
-      <c r="M929"/>
+      <c r="M929" t="s">
+        <v>222</v>
+      </c>
       <c r="N929"/>
       <c r="O929"/>
     </row>
@@ -40005,35 +40072,41 @@
         <v>135</v>
       </c>
       <c r="B930" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C930" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="D930" t="n">
         <v>50</v>
       </c>
-      <c r="E930"/>
+      <c r="E930" t="n">
+        <v>20260810</v>
+      </c>
       <c r="F930" t="n">
-        <v>1257</v>
+        <v>1040</v>
       </c>
       <c r="G930" t="s">
         <v>138</v>
       </c>
       <c r="H930" t="n">
-        <v>4.02</v>
+        <v>5.9</v>
       </c>
       <c r="I930" t="n">
-        <v>4.81</v>
-      </c>
-      <c r="J930"/>
+        <v>47</v>
+      </c>
+      <c r="J930" t="s">
+        <v>176</v>
+      </c>
       <c r="K930" t="n">
-        <v>25.6</v>
+        <v>26</v>
       </c>
       <c r="L930" t="s">
         <v>140</v>
       </c>
-      <c r="M930"/>
+      <c r="M930" t="s">
+        <v>222</v>
+      </c>
       <c r="N930"/>
       <c r="O930"/>
     </row>
@@ -40042,35 +40115,41 @@
         <v>135</v>
       </c>
       <c r="B931" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C931" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D931" t="n">
         <v>15</v>
       </c>
-      <c r="E931"/>
+      <c r="E931" t="n">
+        <v>20260810</v>
+      </c>
       <c r="F931" t="n">
-        <v>919</v>
+        <v>1003</v>
       </c>
       <c r="G931" t="s">
         <v>138</v>
       </c>
       <c r="H931" t="n">
-        <v>5.21</v>
+        <v>6.21</v>
       </c>
       <c r="I931" t="n">
-        <v>3.16</v>
-      </c>
-      <c r="J931"/>
+        <v>24.4</v>
+      </c>
+      <c r="J931" t="s">
+        <v>176</v>
+      </c>
       <c r="K931" t="n">
-        <v>24.7</v>
+        <v>26.6</v>
       </c>
       <c r="L931" t="s">
         <v>140</v>
       </c>
-      <c r="M931"/>
+      <c r="M931" t="s">
+        <v>222</v>
+      </c>
       <c r="N931"/>
       <c r="O931"/>
     </row>
@@ -40079,38 +40158,42 @@
         <v>135</v>
       </c>
       <c r="B932" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C932" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D932" t="n">
-        <v>30</v>
-      </c>
-      <c r="E932"/>
+        <v>50</v>
+      </c>
+      <c r="E932" t="n">
+        <v>20260810</v>
+      </c>
       <c r="F932" t="n">
-        <v>1217</v>
+        <v>934</v>
       </c>
       <c r="G932" t="s">
         <v>138</v>
       </c>
       <c r="H932" t="n">
-        <v>4.46</v>
+        <v>5.44</v>
       </c>
       <c r="I932" t="n">
-        <v>4.19</v>
-      </c>
-      <c r="J932"/>
+        <v>45.9</v>
+      </c>
+      <c r="J932" t="s">
+        <v>176</v>
+      </c>
       <c r="K932" t="n">
-        <v>26.2</v>
+        <v>25.2</v>
       </c>
       <c r="L932" t="s">
-        <v>162</v>
-      </c>
-      <c r="M932"/>
-      <c r="N932" t="s">
+        <v>140</v>
+      </c>
+      <c r="M932" t="s">
         <v>222</v>
       </c>
+      <c r="N932"/>
       <c r="O932"/>
     </row>
     <row r="933">
@@ -40118,7 +40201,7 @@
         <v>135</v>
       </c>
       <c r="B933" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C933" t="s">
         <v>155</v>
@@ -40126,30 +40209,34 @@
       <c r="D933" t="n">
         <v>50</v>
       </c>
-      <c r="E933"/>
+      <c r="E933" t="n">
+        <v>20260810</v>
+      </c>
       <c r="F933" t="n">
-        <v>1236</v>
+        <v>920</v>
       </c>
       <c r="G933" t="s">
         <v>138</v>
       </c>
       <c r="H933" t="n">
-        <v>3.75</v>
+        <v>7.18</v>
       </c>
       <c r="I933" t="n">
-        <v>8.54</v>
-      </c>
-      <c r="J933"/>
+        <v>624</v>
+      </c>
+      <c r="J933" t="s">
+        <v>176</v>
+      </c>
       <c r="K933" t="n">
-        <v>26.4</v>
+        <v>26.2</v>
       </c>
       <c r="L933" t="s">
-        <v>162</v>
-      </c>
-      <c r="M933"/>
-      <c r="N933" t="s">
+        <v>140</v>
+      </c>
+      <c r="M933" t="s">
         <v>222</v>
       </c>
+      <c r="N933"/>
       <c r="O933"/>
     </row>
     <row r="934">
@@ -40157,35 +40244,41 @@
         <v>135</v>
       </c>
       <c r="B934" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C934" t="s">
         <v>137</v>
       </c>
       <c r="D934" t="n">
-        <v>30</v>
-      </c>
-      <c r="E934"/>
+        <v>50</v>
+      </c>
+      <c r="E934" t="n">
+        <v>20260810</v>
+      </c>
       <c r="F934" t="n">
-        <v>1157</v>
+        <v>948</v>
       </c>
       <c r="G934" t="s">
         <v>138</v>
       </c>
       <c r="H934" t="n">
-        <v>3.85</v>
+        <v>5.32</v>
       </c>
       <c r="I934" t="n">
-        <v>4.92</v>
-      </c>
-      <c r="J934"/>
+        <v>32.6</v>
+      </c>
+      <c r="J934" t="s">
+        <v>176</v>
+      </c>
       <c r="K934" t="n">
-        <v>26.2</v>
+        <v>24.9</v>
       </c>
       <c r="L934" t="s">
         <v>140</v>
       </c>
-      <c r="M934"/>
+      <c r="M934" t="s">
+        <v>222</v>
+      </c>
       <c r="N934"/>
       <c r="O934"/>
     </row>
@@ -40194,36 +40287,44 @@
         <v>135</v>
       </c>
       <c r="B935" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="C935" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="D935" t="n">
         <v>50</v>
       </c>
-      <c r="E935"/>
+      <c r="E935" t="n">
+        <v>20260813</v>
+      </c>
       <c r="F935" t="n">
-        <v>1204</v>
+        <v>835</v>
       </c>
       <c r="G935" t="s">
         <v>138</v>
       </c>
       <c r="H935" t="n">
-        <v>4.03</v>
+        <v>6.93</v>
       </c>
       <c r="I935" t="n">
-        <v>4.35</v>
-      </c>
-      <c r="J935"/>
+        <v>124.9</v>
+      </c>
+      <c r="J935" t="s">
+        <v>176</v>
+      </c>
       <c r="K935" t="n">
-        <v>25.5</v>
+        <v>24.9</v>
       </c>
       <c r="L935" t="s">
         <v>140</v>
       </c>
-      <c r="M935"/>
-      <c r="N935"/>
+      <c r="M935" t="s">
+        <v>222</v>
+      </c>
+      <c r="N935" t="s">
+        <v>223</v>
+      </c>
       <c r="O935"/>
     </row>
     <row r="936">
@@ -40231,35 +40332,41 @@
         <v>135</v>
       </c>
       <c r="B936" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C936" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D936" t="n">
         <v>30</v>
       </c>
-      <c r="E936"/>
+      <c r="E936" t="n">
+        <v>20260813</v>
+      </c>
       <c r="F936" t="n">
-        <v>1117</v>
+        <v>820</v>
       </c>
       <c r="G936" t="s">
         <v>138</v>
       </c>
       <c r="H936" t="n">
-        <v>6.48</v>
+        <v>7.08</v>
       </c>
       <c r="I936" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="J936"/>
+        <v>100.1</v>
+      </c>
+      <c r="J936" t="s">
+        <v>176</v>
+      </c>
       <c r="K936" t="n">
-        <v>26.6</v>
+        <v>24.9</v>
       </c>
       <c r="L936" t="s">
         <v>140</v>
       </c>
-      <c r="M936"/>
+      <c r="M936" t="s">
+        <v>222</v>
+      </c>
       <c r="N936"/>
       <c r="O936"/>
     </row>
@@ -40268,36 +40375,44 @@
         <v>135</v>
       </c>
       <c r="B937" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C937" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
       <c r="D937" t="n">
         <v>15</v>
       </c>
-      <c r="E937"/>
+      <c r="E937" t="n">
+        <v>20260813</v>
+      </c>
       <c r="F937" t="n">
-        <v>1111</v>
+        <v>905</v>
       </c>
       <c r="G937" t="s">
         <v>138</v>
       </c>
       <c r="H937" t="n">
-        <v>6.49</v>
+        <v>5.99</v>
       </c>
       <c r="I937" t="n">
-        <v>322</v>
-      </c>
-      <c r="J937"/>
+        <v>1822</v>
+      </c>
+      <c r="J937" t="s">
+        <v>173</v>
+      </c>
       <c r="K937" t="n">
-        <v>24.6</v>
+        <v>24.7</v>
       </c>
       <c r="L937" t="s">
-        <v>140</v>
-      </c>
-      <c r="M937"/>
-      <c r="N937"/>
+        <v>162</v>
+      </c>
+      <c r="M937" t="s">
+        <v>222</v>
+      </c>
+      <c r="N937" t="s">
+        <v>224</v>
+      </c>
       <c r="O937"/>
     </row>
     <row r="938">
@@ -40305,36 +40420,44 @@
         <v>135</v>
       </c>
       <c r="B938" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C938" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="D938" t="n">
-        <v>30</v>
-      </c>
-      <c r="E938"/>
+        <v>15</v>
+      </c>
+      <c r="E938" t="n">
+        <v>20260813</v>
+      </c>
       <c r="F938" t="n">
-        <v>1030</v>
+        <v>851</v>
       </c>
       <c r="G938" t="s">
         <v>138</v>
       </c>
       <c r="H938" t="n">
-        <v>5.83</v>
+        <v>6.18</v>
       </c>
       <c r="I938" t="n">
-        <v>56.6</v>
-      </c>
-      <c r="J938"/>
+        <v>1752</v>
+      </c>
+      <c r="J938" t="s">
+        <v>173</v>
+      </c>
       <c r="K938" t="n">
-        <v>25.3</v>
+        <v>25.2</v>
       </c>
       <c r="L938" t="s">
         <v>140</v>
       </c>
-      <c r="M938"/>
-      <c r="N938"/>
+      <c r="M938" t="s">
+        <v>222</v>
+      </c>
+      <c r="N938" t="s">
+        <v>224</v>
+      </c>
       <c r="O938"/>
     </row>
     <row r="939">
@@ -40342,35 +40465,41 @@
         <v>135</v>
       </c>
       <c r="B939" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C939" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="D939" t="n">
         <v>50</v>
       </c>
-      <c r="E939"/>
+      <c r="E939" t="n">
+        <v>20260813</v>
+      </c>
       <c r="F939" t="n">
-        <v>1040</v>
+        <v>854</v>
       </c>
       <c r="G939" t="s">
         <v>138</v>
       </c>
       <c r="H939" t="n">
-        <v>5.9</v>
+        <v>4.28</v>
       </c>
       <c r="I939" t="n">
-        <v>47</v>
-      </c>
-      <c r="J939"/>
+        <v>6.71</v>
+      </c>
+      <c r="J939" t="s">
+        <v>176</v>
+      </c>
       <c r="K939" t="n">
-        <v>26</v>
+        <v>24.4</v>
       </c>
       <c r="L939" t="s">
         <v>140</v>
       </c>
-      <c r="M939"/>
+      <c r="M939" t="s">
+        <v>222</v>
+      </c>
       <c r="N939"/>
       <c r="O939"/>
     </row>
@@ -40379,35 +40508,41 @@
         <v>135</v>
       </c>
       <c r="B940" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C940" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="D940" t="n">
-        <v>15</v>
-      </c>
-      <c r="E940"/>
+        <v>50</v>
+      </c>
+      <c r="E940" t="n">
+        <v>20260813</v>
+      </c>
       <c r="F940" t="n">
-        <v>1122</v>
+        <v>915</v>
       </c>
       <c r="G940" t="s">
         <v>138</v>
       </c>
       <c r="H940" t="n">
-        <v>6.63</v>
+        <v>4.6</v>
       </c>
       <c r="I940" t="n">
-        <v>67.4</v>
-      </c>
-      <c r="J940"/>
+        <v>3.69</v>
+      </c>
+      <c r="J940" t="s">
+        <v>176</v>
+      </c>
       <c r="K940" t="n">
-        <v>26.2</v>
+        <v>23.9</v>
       </c>
       <c r="L940" t="s">
         <v>140</v>
       </c>
-      <c r="M940"/>
+      <c r="M940" t="s">
+        <v>222</v>
+      </c>
       <c r="N940"/>
       <c r="O940"/>
     </row>
@@ -40416,35 +40551,41 @@
         <v>135</v>
       </c>
       <c r="B941" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C941" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D941" t="n">
         <v>15</v>
       </c>
-      <c r="E941"/>
+      <c r="E941" t="n">
+        <v>20260813</v>
+      </c>
       <c r="F941" t="n">
-        <v>1003</v>
+        <v>919</v>
       </c>
       <c r="G941" t="s">
         <v>138</v>
       </c>
       <c r="H941" t="n">
-        <v>6.21</v>
+        <v>5.21</v>
       </c>
       <c r="I941" t="n">
-        <v>24.4</v>
-      </c>
-      <c r="J941"/>
+        <v>3.16</v>
+      </c>
+      <c r="J941" t="s">
+        <v>176</v>
+      </c>
       <c r="K941" t="n">
-        <v>26.6</v>
+        <v>24.7</v>
       </c>
       <c r="L941" t="s">
         <v>140</v>
       </c>
-      <c r="M941"/>
+      <c r="M941" t="s">
+        <v>222</v>
+      </c>
       <c r="N941"/>
       <c r="O941"/>
     </row>
@@ -40456,32 +40597,38 @@
         <v>141</v>
       </c>
       <c r="C942" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D942" t="n">
-        <v>50</v>
-      </c>
-      <c r="E942"/>
+        <v>30</v>
+      </c>
+      <c r="E942" t="n">
+        <v>20260813</v>
+      </c>
       <c r="F942" t="n">
-        <v>934</v>
+        <v>1117</v>
       </c>
       <c r="G942" t="s">
         <v>138</v>
       </c>
       <c r="H942" t="n">
-        <v>5.44</v>
+        <v>6.48</v>
       </c>
       <c r="I942" t="n">
-        <v>45.9</v>
-      </c>
-      <c r="J942"/>
+        <v>0.1</v>
+      </c>
+      <c r="J942" t="s">
+        <v>176</v>
+      </c>
       <c r="K942" t="n">
-        <v>25.2</v>
+        <v>26.6</v>
       </c>
       <c r="L942" t="s">
         <v>140</v>
       </c>
-      <c r="M942"/>
+      <c r="M942" t="s">
+        <v>222</v>
+      </c>
       <c r="N942"/>
       <c r="O942"/>
     </row>
@@ -40493,32 +40640,38 @@
         <v>141</v>
       </c>
       <c r="C943" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="D943" t="n">
-        <v>50</v>
-      </c>
-      <c r="E943"/>
+        <v>15</v>
+      </c>
+      <c r="E943" t="n">
+        <v>20260813</v>
+      </c>
       <c r="F943" t="n">
-        <v>920</v>
+        <v>1111</v>
       </c>
       <c r="G943" t="s">
         <v>138</v>
       </c>
       <c r="H943" t="n">
-        <v>7.18</v>
+        <v>6.49</v>
       </c>
       <c r="I943" t="n">
-        <v>624</v>
-      </c>
-      <c r="J943"/>
+        <v>322</v>
+      </c>
+      <c r="J943" t="s">
+        <v>176</v>
+      </c>
       <c r="K943" t="n">
-        <v>26.2</v>
+        <v>24.6</v>
       </c>
       <c r="L943" t="s">
         <v>140</v>
       </c>
-      <c r="M943"/>
+      <c r="M943" t="s">
+        <v>222</v>
+      </c>
       <c r="N943"/>
       <c r="O943"/>
     </row>
@@ -40530,32 +40683,38 @@
         <v>141</v>
       </c>
       <c r="C944" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D944" t="n">
-        <v>30</v>
-      </c>
-      <c r="E944"/>
+        <v>15</v>
+      </c>
+      <c r="E944" t="n">
+        <v>20260813</v>
+      </c>
       <c r="F944" t="n">
-        <v>1135</v>
+        <v>1122</v>
       </c>
       <c r="G944" t="s">
         <v>138</v>
       </c>
       <c r="H944" t="n">
-        <v>6.19</v>
+        <v>6.63</v>
       </c>
       <c r="I944" t="n">
-        <v>47.1</v>
-      </c>
-      <c r="J944"/>
+        <v>67.4</v>
+      </c>
+      <c r="J944" t="s">
+        <v>176</v>
+      </c>
       <c r="K944" t="n">
-        <v>25.4</v>
+        <v>26.2</v>
       </c>
       <c r="L944" t="s">
         <v>140</v>
       </c>
-      <c r="M944"/>
+      <c r="M944" t="s">
+        <v>222</v>
+      </c>
       <c r="N944"/>
       <c r="O944"/>
     </row>
@@ -40570,29 +40729,35 @@
         <v>137</v>
       </c>
       <c r="D945" t="n">
-        <v>50</v>
-      </c>
-      <c r="E945"/>
+        <v>30</v>
+      </c>
+      <c r="E945" t="n">
+        <v>20260813</v>
+      </c>
       <c r="F945" t="n">
-        <v>948</v>
+        <v>1135</v>
       </c>
       <c r="G945" t="s">
         <v>138</v>
       </c>
       <c r="H945" t="n">
-        <v>5.32</v>
+        <v>6.19</v>
       </c>
       <c r="I945" t="n">
-        <v>32.6</v>
-      </c>
-      <c r="J945"/>
+        <v>47.1</v>
+      </c>
+      <c r="J945" t="s">
+        <v>176</v>
+      </c>
       <c r="K945" t="n">
-        <v>24.9</v>
+        <v>25.4</v>
       </c>
       <c r="L945" t="s">
         <v>140</v>
       </c>
-      <c r="M945"/>
+      <c r="M945" t="s">
+        <v>222</v>
+      </c>
       <c r="N945"/>
       <c r="O945"/>
     </row>

</xml_diff>